<commit_message>
Admissions audit: add live status of 26 Oct 2025 amendments to annex; English-first reply draft anchored in the existing thread
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PwvPj41jSev9ApGi3qLq4f
</commit_message>
<xml_diff>
--- a/pmu-admissions-audit/final_review/مرفق_التصحيحات_والقرارات_المطلوبة.xlsx
+++ b/pmu-admissions-audit/final_review/مرفق_التصحيحات_والقرارات_المطلوبة.xlsx
@@ -7,15 +7,18 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تصحيحات تحريرية جاهزة" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="قرارات مطلوبة" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملاحظات الإعداد" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حالة تعديلات 26 أكتوبر 2025" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تصحيحات تحريرية جاهزة" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="قرارات مطلوبة" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ملاحظات الإعداد" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'تصحيحات تحريرية جاهزة'!$A$4:$H$52</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'تصحيحات تحريرية جاهزة'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'قرارات مطلوبة'!$A$4:$J$36</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'قرارات مطلوبة'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'حالة تعديلات 26 أكتوبر 2025'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'حالة تعديلات 26 أكتوبر 2025'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'تصحيحات تحريرية جاهزة'!$A$4:$H$52</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'تصحيحات تحريرية جاهزة'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'قرارات مطلوبة'!$A$4:$J$36</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'قرارات مطلوبة'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -145,6 +148,30 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="007F4F00"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -506,6 +533,281 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>حالة التعديلات المطلوبة في رد 26 أكتوبر 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>تحقق مباشر من الموقع الحي بتاريخ 13 أكتوبر 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>التعديل المطلوب في رد 26 أكتوبر 2025</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>الحالة على الموقع (13 أكتوبر 2026)</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>الدليل المنشور (حرفيًا)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>الرابط</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>المطلوب لإغلاقه</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>الحد الأدنى للمجموع الموزون: 74% للحاسب والهندسة، و72% لغير الهندسية، مع ملاحظة المفاضلة والمقابلة الشخصية</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>لم يُنفَّذ</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>HS GPA out of 100 ≥ 85 40% Qudrat ≥ 65 30% Tahseely ≥ 65 30% *Students with lower marks may apply, however, the minimum weighted total, defined by the Admissions Office, should be met.</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>https://www.pmu.edu.sa/admission/admissions_requirements_cs_eng_majors</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>نشر النسبتين المعتمدتين والملاحظة في صفحتي القبول في البكالوريوس ومتطلبات الحاسب والهندسة</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="9" t="inlineStr">
+        <is>
+          <t>إضافة برنامج B.S. Chemical Engineering</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>منفّذ جزئيًا</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>These majors are Architecture, Computer Science, Computer Engineering, Software Engineering, Mechanical Engineering, Electrical Engineering and Civil Engineering.</t>
+        </is>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>https://www.pmu.edu.sa/admission/admissions_requirements_cs_eng_majors</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
+          <t>أُضيف إلى قوائم البرامج، ولم يُضف إلى قائمة التخصصات في صفحتي متطلبات الحاسب والهندسة واختبار SAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>رسم التقديم للطلاب الدوليين والمحولين والزائرين من 500 إلى 950 ريالًا</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>منفّذ جزئيًا</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Pay a non-refundable application fee of SAR 500 (excl. VAT) upon submission of documents</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>https://www.pmu.edu.sa/admission/international_students</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>حُدِّث في صفحتي التحويل والزائرين (950 شاملة الضريبة)، وبقي 500 في صفحة الطلاب الدوليين؛ ويلزم توحيد المعالجة الضريبية: طُلب «excl. VAT» والمنشور «incl. VAT»</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>إزالة اشتراط (SAAT) أو ما يعادله (SAT 2) لتخصصات الحاسب والهندسة</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>منفّذ جزئيًا</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Computer Science &amp; Engineering Majors: Secondary School 40% SAT I 30% SAT II 30%</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>https://www.pmu.edu.sa/admission/international_students</t>
+        </is>
+      </c>
+      <c r="F8" s="9" t="inlineStr">
+        <is>
+          <t>أُزيل SAT 2 من صفحة متطلبات الحاسب والهندسة، وما زال SAT II بوزن 30% في صفحة الطلاب الدوليين</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>رسم إعادة اختبار APTIS من 575 إلى 950 ريالًا (شامل الضريبة)</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>لم يُنفَّذ</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>APTIS Exam Fees SAR 575</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>https://www.pmu.edu.sa/admission/student_fees_tf_ro</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>تحديث جدول الرسوم بعد تأكيد الشؤون المالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>تحديث دليل التقديم الإلكتروني (Web Admission Guide) ليعكس التعديلات</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>لم يُنفَّذ</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>Application Fee SR 500.00 (non refundable)</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>https://www.pmu.edu.sa/Attachments/Admission/Images/PDF/Web-Admission-Guide-v2-2_20-12-18.pdf</t>
+        </is>
+      </c>
+      <c r="F10" s="9" t="inlineStr">
+        <is>
+          <t>استبدال دليل 2018 بدليل محدَّث أو سحبه من القائمة</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F10"/>
+  <conditionalFormatting sqref="C5:C10">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>C5="لم يُنفَّذ"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>C5="منفّذ جزئيًا"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader>&amp;R&amp;8 مرفق سجل ملاحظات صفحات مكتب القبول</oddHeader>
+    <oddFooter>&amp;C&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2521,7 +2823,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3852,7 +4154,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>